<commit_message>
added graphql testcases and updated error storing
</commit_message>
<xml_diff>
--- a/sample_testcases.xlsx
+++ b/sample_testcases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,23 +409,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TC_RESERVATION_001</v>
+        <v>TC_GQL_001</v>
       </c>
       <c r="B2" t="str">
-        <v>{"vehicleId":"v-101","startDate":"2026-08-10","endDate":"2026-08-15","customerName":"John Doe"}</v>
+        <v>{"query":"query GetAllLocations { locations { id name city state } }"}</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TC_RESERVATION_002</v>
+        <v>TC_GQL_002</v>
       </c>
       <c r="B3" t="str">
-        <v>{"vehicleId":"v-102","startDate":"2026-08-12","endDate":"2026-08-18","customerName":"Jane Smith"}</v>
+        <v>{"query":"query GetVehiclesByLocation(: ID!, : String!, : String!) { vehiclesAtLocation(locationId: , startDate: , toDate: ) { id model availableUnits } }","variables":{"locationId":"loc-101","startDate":"2026-09-01","toDate":"2026-09-05"}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_GQL_003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>{"query":"mutation CreateReservation(: ReservationInput!) { createReservation(input: ) { id status confirmationCode } }","variables":{"input":{"vehicleId":"v-101","startDate":"2026-09-01","endDate":"2026-09-05","customerName":"John Doe"}}}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>